<commit_message>
v7.3.85: WorkPackageTable, Login-Fix, ENUM-Erweiterung
</commit_message>
<xml_diff>
--- a/Vorlagen/Arbeitsplan Importdatei Beispiel.xlsx
+++ b/Vorlagen/Arbeitsplan Importdatei Beispiel.xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11214"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10110"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mdbs/Documents/Dev/PZE/Vorlagen/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{061DB886-97CB-EF4B-B99E-DB76EB81B225}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D236C174-EA32-B949-BA9C-21B1B0F0C5AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-18240" yWindow="-23240" windowWidth="25960" windowHeight="16240" xr2:uid="{E8C63C03-1989-034D-A6D2-48A42833948A}"/>
+    <workbookView xWindow="-18240" yWindow="-21000" windowWidth="25960" windowHeight="16240" xr2:uid="{E8C63C03-1989-034D-A6D2-48A42833948A}"/>
   </bookViews>
   <sheets>
     <sheet name="Arbeitsplan import" sheetId="1" r:id="rId1"/>
+    <sheet name="Projektplan" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="185" uniqueCount="82">
   <si>
     <t>Arbeitspakete</t>
   </si>
@@ -144,13 +145,153 @@
   </si>
   <si>
     <t>Musterprojekt</t>
+  </si>
+  <si>
+    <t>MA-Nr
+(gem. lfd. Nr.
+Anl. 6.1 Sp. 1)</t>
+  </si>
+  <si>
+    <t>PM</t>
+  </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t>Anforderungsprofil und Lösungskonzept (alle)</t>
+  </si>
+  <si>
+    <t>01.10.2025</t>
+  </si>
+  <si>
+    <t>30.10.2025</t>
+  </si>
+  <si>
+    <t>03.11.2025</t>
+  </si>
+  <si>
+    <t>30.11.2025</t>
+  </si>
+  <si>
+    <t>01.12.2025</t>
+  </si>
+  <si>
+    <t>31.12.2025</t>
+  </si>
+  <si>
+    <t>1.3.</t>
+  </si>
+  <si>
+    <t>2</t>
+  </si>
+  <si>
+    <t>Entwicklung des Laser- und Lackierverfahrens (Elektra)</t>
+  </si>
+  <si>
+    <t>3</t>
+  </si>
+  <si>
+    <t>Entwicklung von laserfähigem elektrisch leitfähigen Lacksystem (Nordwest-Chemie)</t>
+  </si>
+  <si>
+    <t>4</t>
+  </si>
+  <si>
+    <t>Entwicklung Sensorstruktur, Steuerelektronik und Kontaktierung zwischen Leiterplatte und leitfähigem Lacksystem (Automotive Synergies)</t>
+  </si>
+  <si>
+    <t>4.1</t>
+  </si>
+  <si>
+    <t>Entwicklung der Geometrien und Leiterbahnführung für Sensorflächen in Abhängigkeit der Leitlackparameter (Simulation)</t>
+  </si>
+  <si>
+    <t>04.01.2026</t>
+  </si>
+  <si>
+    <t>26.02.2026</t>
+  </si>
+  <si>
+    <t>01.03.2026</t>
+  </si>
+  <si>
+    <t>31.03.2026</t>
+  </si>
+  <si>
+    <t>01.04.2026</t>
+  </si>
+  <si>
+    <t>31.05.2026</t>
+  </si>
+  <si>
+    <t>01.06.2026</t>
+  </si>
+  <si>
+    <t>31.07.2026</t>
+  </si>
+  <si>
+    <t>4.4</t>
+  </si>
+  <si>
+    <t>Analyse und Auswahl verschiedener Funktionsmustervarianten</t>
+  </si>
+  <si>
+    <t>02.08.2026</t>
+  </si>
+  <si>
+    <t>30.09.2026</t>
+  </si>
+  <si>
+    <t>01.10.2026</t>
+  </si>
+  <si>
+    <t>29.10.2026</t>
+  </si>
+  <si>
+    <t>01.11.2026</t>
+  </si>
+  <si>
+    <t>30.11.2026</t>
+  </si>
+  <si>
+    <t>01.12.2026</t>
+  </si>
+  <si>
+    <t>31.12.2026</t>
+  </si>
+  <si>
+    <t>4.5</t>
+  </si>
+  <si>
+    <t>Entwicklung der Kontaktierung</t>
+  </si>
+  <si>
+    <t>03.01.2027</t>
+  </si>
+  <si>
+    <t>29.04.2027</t>
+  </si>
+  <si>
+    <t>02.05.2027</t>
+  </si>
+  <si>
+    <t>31.08.2027</t>
+  </si>
+  <si>
+    <t>01.09.2027</t>
+  </si>
+  <si>
+    <t>30.09.2027</t>
+  </si>
+  <si>
+    <t>Summe</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -171,6 +312,30 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="3">
@@ -220,10 +385,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -278,9 +444,28 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
+    <cellStyle name="Standard 2" xfId="1" xr:uid="{4C071C3F-3408-604F-8330-982CE1994F3F}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -879,4 +1064,862 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8843646A-9987-9041-9268-B99B324677BF}">
+  <dimension ref="A1:F48"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="14.1640625" defaultRowHeight="18" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="19.6640625" style="22" customWidth="1"/>
+    <col min="2" max="2" width="49.5" style="22" bestFit="1" customWidth="1"/>
+    <col min="3" max="6" width="19.6640625" style="22" customWidth="1"/>
+    <col min="7" max="16384" width="14.1640625" style="22"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" s="19" customFormat="1" ht="95" x14ac:dyDescent="0.2">
+      <c r="A1" s="18" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" s="18" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="18" t="s">
+        <v>4</v>
+      </c>
+      <c r="D1" s="18" t="s">
+        <v>5</v>
+      </c>
+      <c r="E1" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="F1" s="18" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" ht="19" x14ac:dyDescent="0.2">
+      <c r="A2" s="20" t="s">
+        <v>38</v>
+      </c>
+      <c r="B2" s="21" t="s">
+        <v>39</v>
+      </c>
+      <c r="C2" s="20"/>
+      <c r="D2" s="20"/>
+      <c r="E2" s="20"/>
+      <c r="F2" s="20"/>
+    </row>
+    <row r="3" spans="1:6" ht="38" x14ac:dyDescent="0.2">
+      <c r="A3" s="20" t="s">
+        <v>7</v>
+      </c>
+      <c r="B3" s="21" t="s">
+        <v>8</v>
+      </c>
+      <c r="C3" s="20" t="s">
+        <v>40</v>
+      </c>
+      <c r="D3" s="20" t="s">
+        <v>41</v>
+      </c>
+      <c r="E3" s="20">
+        <v>1</v>
+      </c>
+      <c r="F3" s="20">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A4" s="20" t="s">
+        <v>7</v>
+      </c>
+      <c r="B4" s="21"/>
+      <c r="C4" s="20" t="s">
+        <v>40</v>
+      </c>
+      <c r="D4" s="20" t="s">
+        <v>41</v>
+      </c>
+      <c r="E4" s="20">
+        <v>2</v>
+      </c>
+      <c r="F4" s="20">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="19" x14ac:dyDescent="0.2">
+      <c r="A5" s="20" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" s="21" t="s">
+        <v>10</v>
+      </c>
+      <c r="C5" s="20" t="s">
+        <v>42</v>
+      </c>
+      <c r="D5" s="20" t="s">
+        <v>43</v>
+      </c>
+      <c r="E5" s="20">
+        <v>1</v>
+      </c>
+      <c r="F5" s="20">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A6" s="20" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" s="21"/>
+      <c r="C6" s="20" t="s">
+        <v>42</v>
+      </c>
+      <c r="D6" s="20" t="s">
+        <v>43</v>
+      </c>
+      <c r="E6" s="20">
+        <v>2</v>
+      </c>
+      <c r="F6" s="20">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="19" x14ac:dyDescent="0.2">
+      <c r="A7" s="20" t="s">
+        <v>11</v>
+      </c>
+      <c r="B7" s="21" t="s">
+        <v>12</v>
+      </c>
+      <c r="C7" s="20" t="s">
+        <v>44</v>
+      </c>
+      <c r="D7" s="20" t="s">
+        <v>45</v>
+      </c>
+      <c r="E7" s="20">
+        <v>1</v>
+      </c>
+      <c r="F7" s="20">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A8" s="20" t="s">
+        <v>46</v>
+      </c>
+      <c r="B8" s="21"/>
+      <c r="C8" s="20" t="s">
+        <v>44</v>
+      </c>
+      <c r="D8" s="20" t="s">
+        <v>45</v>
+      </c>
+      <c r="E8" s="20">
+        <v>2</v>
+      </c>
+      <c r="F8" s="20">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A9" s="20" t="s">
+        <v>11</v>
+      </c>
+      <c r="B9" s="21"/>
+      <c r="C9" s="20" t="s">
+        <v>44</v>
+      </c>
+      <c r="D9" s="20" t="s">
+        <v>45</v>
+      </c>
+      <c r="E9" s="20">
+        <v>3</v>
+      </c>
+      <c r="F9" s="20">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" ht="38" x14ac:dyDescent="0.2">
+      <c r="A10" s="20" t="s">
+        <v>47</v>
+      </c>
+      <c r="B10" s="21" t="s">
+        <v>48</v>
+      </c>
+      <c r="C10" s="20"/>
+      <c r="D10" s="20"/>
+      <c r="E10" s="20"/>
+      <c r="F10" s="20"/>
+    </row>
+    <row r="11" spans="1:6" ht="38" x14ac:dyDescent="0.2">
+      <c r="A11" s="20" t="s">
+        <v>49</v>
+      </c>
+      <c r="B11" s="21" t="s">
+        <v>50</v>
+      </c>
+      <c r="C11" s="20"/>
+      <c r="D11" s="20"/>
+      <c r="E11" s="20"/>
+      <c r="F11" s="20"/>
+    </row>
+    <row r="12" spans="1:6" ht="76" x14ac:dyDescent="0.2">
+      <c r="A12" s="20" t="s">
+        <v>51</v>
+      </c>
+      <c r="B12" s="21" t="s">
+        <v>52</v>
+      </c>
+      <c r="C12" s="20"/>
+      <c r="D12" s="20"/>
+      <c r="E12" s="20"/>
+      <c r="F12" s="20"/>
+    </row>
+    <row r="13" spans="1:6" ht="76" x14ac:dyDescent="0.2">
+      <c r="A13" s="20" t="s">
+        <v>53</v>
+      </c>
+      <c r="B13" s="21" t="s">
+        <v>54</v>
+      </c>
+      <c r="C13" s="20"/>
+      <c r="D13" s="20"/>
+      <c r="E13" s="20"/>
+      <c r="F13" s="20"/>
+    </row>
+    <row r="14" spans="1:6" ht="76" x14ac:dyDescent="0.2">
+      <c r="A14" s="20" t="s">
+        <v>13</v>
+      </c>
+      <c r="B14" s="21" t="s">
+        <v>14</v>
+      </c>
+      <c r="C14" s="20" t="s">
+        <v>55</v>
+      </c>
+      <c r="D14" s="20" t="s">
+        <v>56</v>
+      </c>
+      <c r="E14" s="20">
+        <v>1</v>
+      </c>
+      <c r="F14" s="20">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A15" s="20" t="s">
+        <v>13</v>
+      </c>
+      <c r="B15" s="21"/>
+      <c r="C15" s="20" t="s">
+        <v>55</v>
+      </c>
+      <c r="D15" s="20" t="s">
+        <v>56</v>
+      </c>
+      <c r="E15" s="20">
+        <v>2</v>
+      </c>
+      <c r="F15" s="20">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A16" s="20" t="s">
+        <v>13</v>
+      </c>
+      <c r="B16" s="21"/>
+      <c r="C16" s="20" t="s">
+        <v>55</v>
+      </c>
+      <c r="D16" s="20" t="s">
+        <v>56</v>
+      </c>
+      <c r="E16" s="20">
+        <v>3</v>
+      </c>
+      <c r="F16" s="20">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" ht="19" x14ac:dyDescent="0.2">
+      <c r="A17" s="20" t="s">
+        <v>15</v>
+      </c>
+      <c r="B17" s="21" t="s">
+        <v>16</v>
+      </c>
+      <c r="C17" s="20" t="s">
+        <v>57</v>
+      </c>
+      <c r="D17" s="20" t="s">
+        <v>58</v>
+      </c>
+      <c r="E17" s="20">
+        <v>1</v>
+      </c>
+      <c r="F17" s="20">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A18" s="20" t="s">
+        <v>15</v>
+      </c>
+      <c r="B18" s="21"/>
+      <c r="C18" s="20" t="s">
+        <v>57</v>
+      </c>
+      <c r="D18" s="20" t="s">
+        <v>58</v>
+      </c>
+      <c r="E18" s="20">
+        <v>2</v>
+      </c>
+      <c r="F18" s="20">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A19" s="20" t="s">
+        <v>15</v>
+      </c>
+      <c r="B19" s="21"/>
+      <c r="C19" s="20" t="s">
+        <v>57</v>
+      </c>
+      <c r="D19" s="20" t="s">
+        <v>58</v>
+      </c>
+      <c r="E19" s="20">
+        <v>3</v>
+      </c>
+      <c r="F19" s="20">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" ht="38" x14ac:dyDescent="0.2">
+      <c r="A20" s="20" t="s">
+        <v>17</v>
+      </c>
+      <c r="B20" s="21" t="s">
+        <v>18</v>
+      </c>
+      <c r="C20" s="20" t="s">
+        <v>59</v>
+      </c>
+      <c r="D20" s="20" t="s">
+        <v>60</v>
+      </c>
+      <c r="E20" s="20">
+        <v>1</v>
+      </c>
+      <c r="F20" s="20">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A21" s="20" t="s">
+        <v>17</v>
+      </c>
+      <c r="B21" s="21"/>
+      <c r="C21" s="20" t="s">
+        <v>59</v>
+      </c>
+      <c r="D21" s="20" t="s">
+        <v>60</v>
+      </c>
+      <c r="E21" s="20">
+        <v>2</v>
+      </c>
+      <c r="F21" s="20">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A22" s="20" t="s">
+        <v>17</v>
+      </c>
+      <c r="B22" s="21"/>
+      <c r="C22" s="20" t="s">
+        <v>59</v>
+      </c>
+      <c r="D22" s="20" t="s">
+        <v>60</v>
+      </c>
+      <c r="E22" s="20">
+        <v>3</v>
+      </c>
+      <c r="F22" s="20">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" ht="19" x14ac:dyDescent="0.2">
+      <c r="A23" s="20" t="s">
+        <v>19</v>
+      </c>
+      <c r="B23" s="21" t="s">
+        <v>20</v>
+      </c>
+      <c r="C23" s="20" t="s">
+        <v>61</v>
+      </c>
+      <c r="D23" s="20" t="s">
+        <v>62</v>
+      </c>
+      <c r="E23" s="20">
+        <v>1</v>
+      </c>
+      <c r="F23" s="20">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A24" s="20" t="s">
+        <v>19</v>
+      </c>
+      <c r="B24" s="21"/>
+      <c r="C24" s="20" t="s">
+        <v>61</v>
+      </c>
+      <c r="D24" s="20" t="s">
+        <v>62</v>
+      </c>
+      <c r="E24" s="20">
+        <v>2</v>
+      </c>
+      <c r="F24" s="20">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A25" s="20" t="s">
+        <v>19</v>
+      </c>
+      <c r="B25" s="21"/>
+      <c r="C25" s="20" t="s">
+        <v>61</v>
+      </c>
+      <c r="D25" s="20" t="s">
+        <v>62</v>
+      </c>
+      <c r="E25" s="20">
+        <v>3</v>
+      </c>
+      <c r="F25" s="20">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" ht="38" x14ac:dyDescent="0.2">
+      <c r="A26" s="20" t="s">
+        <v>63</v>
+      </c>
+      <c r="B26" s="21" t="s">
+        <v>64</v>
+      </c>
+      <c r="C26" s="20"/>
+      <c r="D26" s="20"/>
+      <c r="E26" s="20"/>
+      <c r="F26" s="20"/>
+    </row>
+    <row r="27" spans="1:6" ht="19" x14ac:dyDescent="0.2">
+      <c r="A27" s="20" t="s">
+        <v>21</v>
+      </c>
+      <c r="B27" s="21" t="s">
+        <v>22</v>
+      </c>
+      <c r="C27" s="20" t="s">
+        <v>65</v>
+      </c>
+      <c r="D27" s="20" t="s">
+        <v>66</v>
+      </c>
+      <c r="E27" s="20">
+        <v>1</v>
+      </c>
+      <c r="F27" s="20">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A28" s="20" t="s">
+        <v>21</v>
+      </c>
+      <c r="B28" s="21"/>
+      <c r="C28" s="20" t="s">
+        <v>65</v>
+      </c>
+      <c r="D28" s="20" t="s">
+        <v>66</v>
+      </c>
+      <c r="E28" s="20">
+        <v>2</v>
+      </c>
+      <c r="F28" s="20">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A29" s="20" t="s">
+        <v>21</v>
+      </c>
+      <c r="B29" s="21"/>
+      <c r="C29" s="20" t="s">
+        <v>65</v>
+      </c>
+      <c r="D29" s="20" t="s">
+        <v>66</v>
+      </c>
+      <c r="E29" s="20">
+        <v>3</v>
+      </c>
+      <c r="F29" s="20">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" ht="38" x14ac:dyDescent="0.2">
+      <c r="A30" s="20" t="s">
+        <v>23</v>
+      </c>
+      <c r="B30" s="21" t="s">
+        <v>24</v>
+      </c>
+      <c r="C30" s="20" t="s">
+        <v>67</v>
+      </c>
+      <c r="D30" s="20" t="s">
+        <v>68</v>
+      </c>
+      <c r="E30" s="20">
+        <v>1</v>
+      </c>
+      <c r="F30" s="20">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A31" s="20" t="s">
+        <v>23</v>
+      </c>
+      <c r="B31" s="21"/>
+      <c r="C31" s="20" t="s">
+        <v>67</v>
+      </c>
+      <c r="D31" s="20" t="s">
+        <v>68</v>
+      </c>
+      <c r="E31" s="20">
+        <v>2</v>
+      </c>
+      <c r="F31" s="20">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A32" s="20"/>
+      <c r="B32" s="21"/>
+      <c r="C32" s="20" t="s">
+        <v>67</v>
+      </c>
+      <c r="D32" s="20" t="s">
+        <v>68</v>
+      </c>
+      <c r="E32" s="20">
+        <v>3</v>
+      </c>
+      <c r="F32" s="20">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" ht="38" x14ac:dyDescent="0.2">
+      <c r="A33" s="20" t="s">
+        <v>25</v>
+      </c>
+      <c r="B33" s="21" t="s">
+        <v>26</v>
+      </c>
+      <c r="C33" s="20" t="s">
+        <v>69</v>
+      </c>
+      <c r="D33" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="E33" s="20">
+        <v>1</v>
+      </c>
+      <c r="F33" s="20">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A34" s="20"/>
+      <c r="B34" s="21"/>
+      <c r="C34" s="20" t="s">
+        <v>69</v>
+      </c>
+      <c r="D34" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="E34" s="20">
+        <v>2</v>
+      </c>
+      <c r="F34" s="20">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A35" s="20"/>
+      <c r="B35" s="21"/>
+      <c r="C35" s="20" t="s">
+        <v>69</v>
+      </c>
+      <c r="D35" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="E35" s="20">
+        <v>3</v>
+      </c>
+      <c r="F35" s="20">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" ht="38" x14ac:dyDescent="0.2">
+      <c r="A36" s="20" t="s">
+        <v>27</v>
+      </c>
+      <c r="B36" s="21" t="s">
+        <v>28</v>
+      </c>
+      <c r="C36" s="20" t="s">
+        <v>71</v>
+      </c>
+      <c r="D36" s="20" t="s">
+        <v>72</v>
+      </c>
+      <c r="E36" s="20">
+        <v>1</v>
+      </c>
+      <c r="F36" s="20">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A37" s="20" t="s">
+        <v>27</v>
+      </c>
+      <c r="B37" s="21"/>
+      <c r="C37" s="20" t="s">
+        <v>71</v>
+      </c>
+      <c r="D37" s="20" t="s">
+        <v>72</v>
+      </c>
+      <c r="E37" s="20">
+        <v>2</v>
+      </c>
+      <c r="F37" s="20">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A38" s="20" t="s">
+        <v>27</v>
+      </c>
+      <c r="B38" s="21"/>
+      <c r="C38" s="20" t="s">
+        <v>71</v>
+      </c>
+      <c r="D38" s="20" t="s">
+        <v>72</v>
+      </c>
+      <c r="E38" s="20">
+        <v>3</v>
+      </c>
+      <c r="F38" s="20">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" ht="19" x14ac:dyDescent="0.2">
+      <c r="A39" s="20" t="s">
+        <v>73</v>
+      </c>
+      <c r="B39" s="21" t="s">
+        <v>74</v>
+      </c>
+      <c r="C39" s="20"/>
+      <c r="D39" s="20"/>
+      <c r="E39" s="20"/>
+      <c r="F39" s="20"/>
+    </row>
+    <row r="40" spans="1:6" ht="57" x14ac:dyDescent="0.2">
+      <c r="A40" s="20" t="s">
+        <v>29</v>
+      </c>
+      <c r="B40" s="21" t="s">
+        <v>30</v>
+      </c>
+      <c r="C40" s="20" t="s">
+        <v>75</v>
+      </c>
+      <c r="D40" s="20" t="s">
+        <v>76</v>
+      </c>
+      <c r="E40" s="20">
+        <v>1</v>
+      </c>
+      <c r="F40" s="20">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A41" s="20" t="s">
+        <v>29</v>
+      </c>
+      <c r="B41" s="21"/>
+      <c r="C41" s="20" t="s">
+        <v>75</v>
+      </c>
+      <c r="D41" s="20" t="s">
+        <v>76</v>
+      </c>
+      <c r="E41" s="20">
+        <v>2</v>
+      </c>
+      <c r="F41" s="20">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A42" s="20" t="s">
+        <v>29</v>
+      </c>
+      <c r="B42" s="21"/>
+      <c r="C42" s="20" t="s">
+        <v>75</v>
+      </c>
+      <c r="D42" s="20" t="s">
+        <v>76</v>
+      </c>
+      <c r="E42" s="20">
+        <v>3</v>
+      </c>
+      <c r="F42" s="20">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" ht="19" x14ac:dyDescent="0.2">
+      <c r="A43" s="20" t="s">
+        <v>31</v>
+      </c>
+      <c r="B43" s="21" t="s">
+        <v>32</v>
+      </c>
+      <c r="C43" s="20" t="s">
+        <v>77</v>
+      </c>
+      <c r="D43" s="20" t="s">
+        <v>78</v>
+      </c>
+      <c r="E43" s="20">
+        <v>1</v>
+      </c>
+      <c r="F43" s="20">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A44" s="20" t="s">
+        <v>31</v>
+      </c>
+      <c r="B44" s="21"/>
+      <c r="C44" s="20" t="s">
+        <v>77</v>
+      </c>
+      <c r="D44" s="20" t="s">
+        <v>78</v>
+      </c>
+      <c r="E44" s="20">
+        <v>2</v>
+      </c>
+      <c r="F44" s="20">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" ht="38" x14ac:dyDescent="0.2">
+      <c r="A45" s="20" t="s">
+        <v>6</v>
+      </c>
+      <c r="B45" s="21" t="s">
+        <v>33</v>
+      </c>
+      <c r="C45" s="20" t="s">
+        <v>79</v>
+      </c>
+      <c r="D45" s="20" t="s">
+        <v>80</v>
+      </c>
+      <c r="E45" s="20">
+        <v>1</v>
+      </c>
+      <c r="F45" s="20">
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A46" s="20" t="s">
+        <v>6</v>
+      </c>
+      <c r="B46" s="21"/>
+      <c r="C46" s="20" t="s">
+        <v>79</v>
+      </c>
+      <c r="D46" s="20" t="s">
+        <v>80</v>
+      </c>
+      <c r="E46" s="20">
+        <v>2</v>
+      </c>
+      <c r="F46" s="20">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A47" s="20" t="s">
+        <v>6</v>
+      </c>
+      <c r="B47" s="21"/>
+      <c r="C47" s="20" t="s">
+        <v>79</v>
+      </c>
+      <c r="D47" s="20" t="s">
+        <v>80</v>
+      </c>
+      <c r="E47" s="20">
+        <v>3</v>
+      </c>
+      <c r="F47" s="20">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A48" s="23"/>
+      <c r="B48" s="23"/>
+      <c r="C48" s="23"/>
+      <c r="D48" s="23"/>
+      <c r="E48" s="24" t="s">
+        <v>81</v>
+      </c>
+      <c r="F48" s="25">
+        <f>SUM(F2:F47)</f>
+        <v>42.75</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+</worksheet>
 </file>
</xml_diff>